<commit_message>
fix: parse 천만-unit premiums and seed resumed Supabase
P now keeps 3.8억 / 4억8,900 / 4억6천만원 instead of truncating to 억. Free-tier pause still needs a keepalive ping or Pro.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/archive/golden/260823/zone_rollup_260823.xlsx
+++ b/data/archive/golden/260823/zone_rollup_260823.xlsx
@@ -587,17 +587,17 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.5~12.5</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -674,17 +674,17 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -761,17 +761,17 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.2</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.2~16</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -848,17 +848,17 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6~10</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -935,17 +935,17 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.8</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.9~12</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1022,17 +1022,17 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.8</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.8</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.8~10.7</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1109,17 +1109,17 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.35</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.58~9.3</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1196,17 +1196,17 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13~14.5</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1283,17 +1283,17 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1370,17 +1370,17 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1457,17 +1457,17 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.8</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.8~27</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20~33</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1631,17 +1631,17 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21~31</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1718,17 +1718,17 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.48</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11~13</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1805,17 +1805,17 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.62</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1892,17 +1892,17 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.7</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.7~23</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1979,17 +1979,17 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>34</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>25~36</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2061,22 +2061,22 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13300억</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6~7.3</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2101,12 +2101,12 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13300</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13300</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -2153,17 +2153,17 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2235,22 +2235,22 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>3억</t>
+          <t>3.8억</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.87</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.5~14</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2275,12 +2275,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
@@ -2327,17 +2327,17 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.06</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.8~7.06</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2414,17 +2414,17 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.85</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16.5</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>15.85~16.5</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2501,17 +2501,17 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.17</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.52</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.17~10.52</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2588,17 +2588,17 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>16.9</t>
+          <t>16.1</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>17.9</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>17~18</t>
+          <t>17~20</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2675,17 +2675,17 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2762,17 +2762,17 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>15.8</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>13.5</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>17.5~18</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2849,17 +2849,17 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>10.25</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.5~12.5</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2936,17 +2936,17 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>12.55</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11.5~12.55</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -3023,17 +3023,17 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>6.8~8</t>
+          <t>2.5~4.1</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -3110,17 +3110,17 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>12~14.2</t>
+          <t>10~13.5</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -3197,17 +3197,17 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>10~11</t>
+          <t>10~12</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -3284,17 +3284,17 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>8.6</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.5~8.6</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3371,17 +3371,17 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9.6</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8~9.6</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.9~4</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -3545,17 +3545,17 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.8~3.9</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3632,17 +3632,17 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>10.65</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>23.5</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>9.9~11</t>
+          <t>13.5~24</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3714,22 +3714,22 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.7억</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>24.85</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.3~37</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3754,12 +3754,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.7</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12.7</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
@@ -3806,17 +3806,17 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>16.86</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>16.86~19</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>10.4~12억</t>
+          <t>10.6~12억</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3898,12 +3898,12 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>13.61</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.5~23.6</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -3980,17 +3980,17 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11.8</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16.4</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>13~18</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -4067,17 +4067,17 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>5.98</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.5~6.2</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -4154,17 +4154,17 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>5.25</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7~8</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -4241,17 +4241,17 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11~13</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -4328,17 +4328,17 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>9.7</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>11~13.2</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -4415,17 +4415,17 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14.2</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>13.5~14</t>
+          <t>12~14.2</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4502,17 +4502,17 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>7.9~8</t>
+          <t>7~9.8</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -4589,17 +4589,17 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>11.7</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>14~16</t>
+          <t>7.5~20</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -4676,17 +4676,17 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>7.9</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>6.5~8</t>
+          <t>4.5~8.1</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4763,17 +4763,17 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>13.3</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>14.5~75</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4850,17 +4850,17 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>12~19</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4937,17 +4937,17 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.5~10</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -5024,17 +5024,17 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2.9</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.1~3.9</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -5106,22 +5106,22 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>4억</t>
+          <t>4.68억</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7.58</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.29~9.5</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -5146,12 +5146,12 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr">
@@ -5193,29 +5193,29 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>4억</t>
+          <t>4.6억</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
+          <t>7.6</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>7.3~8.3</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
           <t>7.6</t>
@@ -5233,12 +5233,12 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr">
@@ -5280,22 +5280,22 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>4.7억</t>
+          <t>4.05~4.7억</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>7.5~8.6</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.05</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">

</xml_diff>